<commit_message>
Labs 2.2.0 - actualizar Maestro (2026-10-15 18:32:02 UTC)
</commit_message>
<xml_diff>
--- a/data/Maestro_Productos_Grido.xlsx
+++ b/data/Maestro_Productos_Grido.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" r:id="R48fa539953c94e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliases" sheetId="2" r:id="R62cbfaac9a0044f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusiones" sheetId="3" r:id="Rdbcf6897d7b64599"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="R690463164d484b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="5" r:id="Rf949728835aa4b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" r:id="R747e6d6964c24753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliases" sheetId="2" r:id="Rb0507c26604d42a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusiones" sheetId="3" r:id="R7789cc705f72416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="Rddf0d05bc2d94fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="5" r:id="R3d919bdf8b4b479a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1319,7 +1319,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1379,6 +1379,13 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1602,13 +1609,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="32.880001068115234" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="36.380001068115234" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="44" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="15.25" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15.5" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="7.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="21.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="8" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -3900,6 +3907,32 @@
       </x:c>
       <x:c r="H95" s="2" t="str">
         <x:v>Agregado 2026-09-03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="B96" s="2" t="n">
+        <x:v>4000993</x:v>
+      </x:c>
+      <x:c r="C96" s="2" t="str">
+        <x:v>PACK 6 CAJAS BOMB CHOCO AVE X8 GR</x:v>
+      </x:c>
+      <x:c r="D96" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E96" s="2" t="str">
+        <x:v>Fraccionable</x:v>
+      </x:c>
+      <x:c r="F96" s="2" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="G96" s="2" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H96" s="2" t="str">
+        <x:v>Agregado por nuevo Mix de Ventas</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3918,7 +3951,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27d4931d53a44fc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19704c9ed6704e68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3927,15 +3960,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="36.75" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="32.880001068115234" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="45" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.630000114440918" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="25.75" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11.75" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="21.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="8.130000114440918" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="16.6299991607666" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" customHeight="1">
@@ -9614,6 +9647,1398 @@
       </x:c>
       <x:c r="I222" s="2" t="str">
         <x:v>Agregado 2026-09-03</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" s="2" t="str">
+        <x:v>Bombon Choco Avellanadas Caja x 8 Un.</x:v>
+      </x:c>
+      <x:c r="B223" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C223" s="2" t="str">
+        <x:v>Caja/pack x8</x:v>
+      </x:c>
+      <x:c r="D223" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E223" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F223" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G223" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H223" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I223" s="2" t="str">
+        <x:v>Compatibilidad nombre actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" s="2" t="str">
+        <x:v>Bombon Choco Avellanadas x Unidad</x:v>
+      </x:c>
+      <x:c r="B224" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C224" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D224" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E224" s="2" t="str">
+        <x:v>cantidad / 8</x:v>
+      </x:c>
+      <x:c r="F224" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G224" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H224" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I224" s="2" t="str">
+        <x:v>Compatibilidad nombre actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" s="2" t="str">
+        <x:v>Bombon Choco Avellanas Caja x 8 Un.</x:v>
+      </x:c>
+      <x:c r="B225" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C225" s="2" t="str">
+        <x:v>Caja/pack x8</x:v>
+      </x:c>
+      <x:c r="D225" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E225" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F225" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G225" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H225" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I225" s="2" t="str">
+        <x:v>Preparado para corrección de nombre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" s="2" t="str">
+        <x:v>Bombon Choco Avellanas x Unidad</x:v>
+      </x:c>
+      <x:c r="B226" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C226" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D226" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E226" s="2" t="str">
+        <x:v>cantidad / 8</x:v>
+      </x:c>
+      <x:c r="F226" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G226" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H226" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I226" s="2" t="str">
+        <x:v>Preparado para corrección de nombre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" s="2" t="str">
+        <x:v>Bombon Choco Avellanadas Caja x 8 Un.</x:v>
+      </x:c>
+      <x:c r="B227" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C227" s="2" t="str">
+        <x:v>Caja/pack x8</x:v>
+      </x:c>
+      <x:c r="D227" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E227" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F227" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G227" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H227" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I227" s="2" t="str">
+        <x:v>Compatibilidad nombre actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" s="2" t="str">
+        <x:v>Bombon Choco Avellanadas x Unidad</x:v>
+      </x:c>
+      <x:c r="B228" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C228" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D228" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E228" s="2" t="str">
+        <x:v>cantidad / 8</x:v>
+      </x:c>
+      <x:c r="F228" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G228" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H228" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I228" s="2" t="str">
+        <x:v>Compatibilidad nombre actual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="A229" s="2" t="str">
+        <x:v>Bombon Choco Avellanas Caja x 8 Un.</x:v>
+      </x:c>
+      <x:c r="B229" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C229" s="2" t="str">
+        <x:v>Caja/pack x8</x:v>
+      </x:c>
+      <x:c r="D229" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E229" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F229" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G229" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H229" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I229" s="2" t="str">
+        <x:v>Preparado para corrección de nombre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="A230" s="2" t="str">
+        <x:v>Bombon Choco Avellanas x Unidad</x:v>
+      </x:c>
+      <x:c r="B230" s="2" t="str">
+        <x:v>bombon choco avellanas</x:v>
+      </x:c>
+      <x:c r="C230" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D230" s="2" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E230" s="2" t="str">
+        <x:v>cantidad / 8</x:v>
+      </x:c>
+      <x:c r="F230" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G230" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H230" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I230" s="2" t="str">
+        <x:v>Preparado para corrección de nombre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" s="2" t="str">
+        <x:v>Alfajor Cookies and Cream x 6u.</x:v>
+      </x:c>
+      <x:c r="B231" s="2" t="str">
+        <x:v>alfajor secreto cookies and cream</x:v>
+      </x:c>
+      <x:c r="C231" s="2" t="str">
+        <x:v>Caja/pack x6</x:v>
+      </x:c>
+      <x:c r="D231" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E231" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F231" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G231" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H231" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I231" s="2" t="str">
+        <x:v>Nuevo nombre Mix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" s="2" t="str">
+        <x:v>Alfajor Cookies and Cream x Un.</x:v>
+      </x:c>
+      <x:c r="B232" s="2" t="str">
+        <x:v>alfajor secreto cookies and cream</x:v>
+      </x:c>
+      <x:c r="C232" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D232" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E232" s="2" t="str">
+        <x:v>cantidad / 6</x:v>
+      </x:c>
+      <x:c r="F232" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G232" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H232" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I232" s="2" t="str">
+        <x:v>Nuevo nombre Mix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" s="2" t="str">
+        <x:v>Alfajor Cookies and Cream x 6u.</x:v>
+      </x:c>
+      <x:c r="B233" s="2" t="str">
+        <x:v>alfajor secreto cookies and cream</x:v>
+      </x:c>
+      <x:c r="C233" s="2" t="str">
+        <x:v>Caja/pack x6</x:v>
+      </x:c>
+      <x:c r="D233" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E233" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F233" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G233" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H233" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I233" s="2" t="str">
+        <x:v>Nuevo nombre Mix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" s="2" t="str">
+        <x:v>Alfajor Cookies and Cream x Un.</x:v>
+      </x:c>
+      <x:c r="B234" s="2" t="str">
+        <x:v>alfajor secreto cookies and cream</x:v>
+      </x:c>
+      <x:c r="C234" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D234" s="2" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E234" s="2" t="str">
+        <x:v>cantidad / 6</x:v>
+      </x:c>
+      <x:c r="F234" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G234" s="2" t="str">
+        <x:v>Bombones</x:v>
+      </x:c>
+      <x:c r="H234" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I234" s="2" t="str">
+        <x:v>Nuevo nombre Mix</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" s="2" t="str">
+        <x:v>Hsaa Chocolate S/Tacc X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B235" s="2" t="str">
+        <x:v>hel dul equi choco 80 gr</x:v>
+      </x:c>
+      <x:c r="C235" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D235" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E235" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F235" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G235" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H235" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I235" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" s="2" t="str">
+        <x:v>Hsaa Chocolate S/Tacc X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B236" s="2" t="str">
+        <x:v>hel dul equi choco 80 gr</x:v>
+      </x:c>
+      <x:c r="C236" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D236" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E236" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F236" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G236" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H236" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I236" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" s="2" t="str">
+        <x:v>Hsaa Frutilla A La Crema S/Tacc X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B237" s="2" t="str">
+        <x:v>hel dul equi fruti 80 gr</x:v>
+      </x:c>
+      <x:c r="C237" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D237" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E237" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F237" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G237" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H237" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I237" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="238">
+      <x:c r="A238" s="2" t="str">
+        <x:v>Hsaa Frutilla A La Crema S/Tacc X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B238" s="2" t="str">
+        <x:v>hel dul equi fruti 80 gr</x:v>
+      </x:c>
+      <x:c r="C238" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D238" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E238" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F238" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G238" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H238" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I238" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="239">
+      <x:c r="A239" s="2" t="str">
+        <x:v>Hsaa Dulce De Leche S/Tacc X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B239" s="2" t="str">
+        <x:v>hel dul equi ddl 80 gr</x:v>
+      </x:c>
+      <x:c r="C239" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D239" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E239" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F239" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G239" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H239" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I239" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="240">
+      <x:c r="A240" s="2" t="str">
+        <x:v>Hsaa Dulce De Leche S/Tacc X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B240" s="2" t="str">
+        <x:v>hel dul equi ddl 80 gr</x:v>
+      </x:c>
+      <x:c r="C240" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D240" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E240" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F240" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G240" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H240" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I240" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="241">
+      <x:c r="A241" s="2" t="str">
+        <x:v>Postre Vegano Chocolate X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B241" s="2" t="str">
+        <x:v>postre veg chocolate 80 gr</x:v>
+      </x:c>
+      <x:c r="C241" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D241" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E241" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F241" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G241" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H241" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I241" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="242">
+      <x:c r="A242" s="2" t="str">
+        <x:v>Postre Vegano Chocolate X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B242" s="2" t="str">
+        <x:v>postre veg chocolate 80 gr</x:v>
+      </x:c>
+      <x:c r="C242" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D242" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E242" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F242" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G242" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H242" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I242" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="243">
+      <x:c r="A243" s="2" t="str">
+        <x:v>Postre Vegano Mani X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B243" s="2" t="str">
+        <x:v>postre veg mani 80 gr</x:v>
+      </x:c>
+      <x:c r="C243" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D243" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E243" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F243" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G243" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H243" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I243" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="244">
+      <x:c r="A244" s="2" t="str">
+        <x:v>Postre Vegano Mani X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B244" s="2" t="str">
+        <x:v>postre veg mani 80 gr</x:v>
+      </x:c>
+      <x:c r="C244" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D244" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E244" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F244" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G244" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H244" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I244" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="245">
+      <x:c r="A245" s="2" t="str">
+        <x:v>Postre Vegano Vanilla X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B245" s="2" t="str">
+        <x:v>postre veg vainilla 80 gr</x:v>
+      </x:c>
+      <x:c r="C245" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D245" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E245" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F245" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G245" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H245" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I245" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="246">
+      <x:c r="A246" s="2" t="str">
+        <x:v>Postre Vegano Vanilla X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B246" s="2" t="str">
+        <x:v>postre veg vainilla 80 gr</x:v>
+      </x:c>
+      <x:c r="C246" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D246" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E246" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F246" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G246" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H246" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I246" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="247">
+      <x:c r="A247" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Frutilla X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B247" s="2" t="str">
+        <x:v>yogurt hel frutilla</x:v>
+      </x:c>
+      <x:c r="C247" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D247" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E247" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F247" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G247" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H247" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I247" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="248">
+      <x:c r="A248" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Frutilla X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B248" s="2" t="str">
+        <x:v>yogurt hel frutilla</x:v>
+      </x:c>
+      <x:c r="C248" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D248" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E248" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F248" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G248" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H248" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I248" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="249">
+      <x:c r="A249" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Mango/Maracuya X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B249" s="2" t="str">
+        <x:v>yogurt hel mango maracuya</x:v>
+      </x:c>
+      <x:c r="C249" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D249" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E249" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F249" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G249" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H249" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I249" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="250">
+      <x:c r="A250" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Mango/Maracuya X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B250" s="2" t="str">
+        <x:v>yogurt hel mango maracuya</x:v>
+      </x:c>
+      <x:c r="C250" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D250" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E250" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F250" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G250" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H250" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I250" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="251">
+      <x:c r="A251" s="2" t="str">
+        <x:v>Yogur S/Tacc Helado Frutos Del Bosque X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B251" s="2" t="str">
+        <x:v>yogurt hel frutos del bosque</x:v>
+      </x:c>
+      <x:c r="C251" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D251" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E251" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F251" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G251" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H251" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I251" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="252">
+      <x:c r="A252" s="2" t="str">
+        <x:v>Yogur S/Tacc Helado Frutos Del Bosque X 12 Unid.</x:v>
+      </x:c>
+      <x:c r="B252" s="2" t="str">
+        <x:v>yogurt hel frutos del bosque</x:v>
+      </x:c>
+      <x:c r="C252" s="2" t="str">
+        <x:v>Caja/pack x12</x:v>
+      </x:c>
+      <x:c r="D252" s="2" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E252" s="2" t="str">
+        <x:v>cantidad * 12</x:v>
+      </x:c>
+      <x:c r="F252" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G252" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H252" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I252" s="2" t="str">
+        <x:v>1 registro x12 = 12 unidades</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="253">
+      <x:c r="A253" s="2" t="str">
+        <x:v>Hsaa Chocolate S/Tacc x Un.</x:v>
+      </x:c>
+      <x:c r="B253" s="2" t="str">
+        <x:v>hel dul equi choco 80 gr</x:v>
+      </x:c>
+      <x:c r="C253" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D253" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E253" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F253" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G253" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H253" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I253" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="254">
+      <x:c r="A254" s="2" t="str">
+        <x:v>Hsaa Chocolate S/Tacc x Un.</x:v>
+      </x:c>
+      <x:c r="B254" s="2" t="str">
+        <x:v>hel dul equi choco 80 gr</x:v>
+      </x:c>
+      <x:c r="C254" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D254" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E254" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F254" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G254" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H254" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I254" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="255">
+      <x:c r="A255" s="2" t="str">
+        <x:v>Hsaa Frutilla A La Crema S/Tacc x Un.</x:v>
+      </x:c>
+      <x:c r="B255" s="2" t="str">
+        <x:v>hel dul equi fruti 80 gr</x:v>
+      </x:c>
+      <x:c r="C255" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D255" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E255" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F255" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G255" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H255" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I255" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="256">
+      <x:c r="A256" s="2" t="str">
+        <x:v>Hsaa Frutilla A La Crema S/Tacc x Un.</x:v>
+      </x:c>
+      <x:c r="B256" s="2" t="str">
+        <x:v>hel dul equi fruti 80 gr</x:v>
+      </x:c>
+      <x:c r="C256" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D256" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E256" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F256" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G256" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H256" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I256" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="A257" s="2" t="str">
+        <x:v>Hsaa Dulce De Leche S/Tacc x Un.</x:v>
+      </x:c>
+      <x:c r="B257" s="2" t="str">
+        <x:v>hel dul equi ddl 80 gr</x:v>
+      </x:c>
+      <x:c r="C257" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D257" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E257" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F257" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G257" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H257" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I257" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="A258" s="2" t="str">
+        <x:v>Hsaa Dulce De Leche S/Tacc x Un.</x:v>
+      </x:c>
+      <x:c r="B258" s="2" t="str">
+        <x:v>hel dul equi ddl 80 gr</x:v>
+      </x:c>
+      <x:c r="C258" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D258" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E258" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F258" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G258" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H258" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I258" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="A259" s="2" t="str">
+        <x:v>Postre Vegano Chocolate x Unidad</x:v>
+      </x:c>
+      <x:c r="B259" s="2" t="str">
+        <x:v>postre veg chocolate 80 gr</x:v>
+      </x:c>
+      <x:c r="C259" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D259" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E259" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F259" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G259" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H259" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I259" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="A260" s="2" t="str">
+        <x:v>Postre Vegano Chocolate x Unidad</x:v>
+      </x:c>
+      <x:c r="B260" s="2" t="str">
+        <x:v>postre veg chocolate 80 gr</x:v>
+      </x:c>
+      <x:c r="C260" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D260" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E260" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F260" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G260" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H260" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I260" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="261">
+      <x:c r="A261" s="2" t="str">
+        <x:v>Postre Vegano Mani x Un.</x:v>
+      </x:c>
+      <x:c r="B261" s="2" t="str">
+        <x:v>postre veg mani 80 gr</x:v>
+      </x:c>
+      <x:c r="C261" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D261" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E261" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F261" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G261" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H261" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I261" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="A262" s="2" t="str">
+        <x:v>Postre Vegano Mani x Un.</x:v>
+      </x:c>
+      <x:c r="B262" s="2" t="str">
+        <x:v>postre veg mani 80 gr</x:v>
+      </x:c>
+      <x:c r="C262" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D262" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E262" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F262" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G262" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H262" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I262" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="263">
+      <x:c r="A263" s="2" t="str">
+        <x:v>Postre Vegano Vanilla x Un.</x:v>
+      </x:c>
+      <x:c r="B263" s="2" t="str">
+        <x:v>postre veg vainilla 80 gr</x:v>
+      </x:c>
+      <x:c r="C263" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D263" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E263" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F263" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G263" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H263" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I263" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="A264" s="2" t="str">
+        <x:v>Postre Vegano Vanilla x Un.</x:v>
+      </x:c>
+      <x:c r="B264" s="2" t="str">
+        <x:v>postre veg vainilla 80 gr</x:v>
+      </x:c>
+      <x:c r="C264" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D264" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E264" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F264" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G264" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H264" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I264" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="A265" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Frutilla x Un.</x:v>
+      </x:c>
+      <x:c r="B265" s="2" t="str">
+        <x:v>yogurt hel frutilla</x:v>
+      </x:c>
+      <x:c r="C265" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D265" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E265" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F265" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G265" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H265" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I265" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="A266" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Frutilla x Un.</x:v>
+      </x:c>
+      <x:c r="B266" s="2" t="str">
+        <x:v>yogurt hel frutilla</x:v>
+      </x:c>
+      <x:c r="C266" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D266" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E266" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F266" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G266" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H266" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I266" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="267">
+      <x:c r="A267" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Mango/Maracuya x Un.</x:v>
+      </x:c>
+      <x:c r="B267" s="2" t="str">
+        <x:v>yogurt hel mango maracuya</x:v>
+      </x:c>
+      <x:c r="C267" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D267" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E267" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F267" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G267" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H267" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I267" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="268">
+      <x:c r="A268" s="2" t="str">
+        <x:v>Yogur Helado S/Tacc Mango/Maracuya x Un.</x:v>
+      </x:c>
+      <x:c r="B268" s="2" t="str">
+        <x:v>yogurt hel mango maracuya</x:v>
+      </x:c>
+      <x:c r="C268" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D268" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E268" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F268" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G268" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H268" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I268" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="A269" s="2" t="str">
+        <x:v>Yogur S/Tacc Helado Frutos Del Bosque x Un.</x:v>
+      </x:c>
+      <x:c r="B269" s="2" t="str">
+        <x:v>yogurt hel frutos del bosque</x:v>
+      </x:c>
+      <x:c r="C269" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D269" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E269" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F269" s="2" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G269" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H269" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I269" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="270">
+      <x:c r="A270" s="2" t="str">
+        <x:v>Yogur S/Tacc Helado Frutos Del Bosque x Un.</x:v>
+      </x:c>
+      <x:c r="B270" s="2" t="str">
+        <x:v>yogurt hel frutos del bosque</x:v>
+      </x:c>
+      <x:c r="C270" s="2" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="D270" s="2" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E270" s="2" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F270" s="2" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G270" s="2" t="str">
+        <x:v>Líneas Especiales C. Heladas</x:v>
+      </x:c>
+      <x:c r="H270" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I270" s="2" t="str">
+        <x:v>Preparado para venta individual</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9632,7 +11057,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bf02caf70644b10"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79ba85ba15ed49cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9641,8 +11066,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <x:cols>
-    <x:col min="1" max="1" width="24.6299991607666" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="33.25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="60" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" customHeight="1">
@@ -9781,10 +11206,434 @@
         <x:v>Omitido por decisión de Gabriel 2026-09-03</x:v>
       </x:c>
     </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="str">
+        <x:v>alfajor cookies and cream uy</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="str">
+        <x:v>Uruguay: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="str">
+        <x:v>hsaa crema con durazno s tacc unid</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="str">
+        <x:v>Producto excluido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="str">
+        <x:v>mix p tacos x conosud</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="str">
+        <x:v>mix para tarta espinaca x 1kg conosud</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="str">
+        <x:v>mix wok de vegetales conosud</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="str">
+        <x:v>papas mccain noisette gr</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="str">
+        <x:v>pimiento morron rojo x 1kg conosud</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="str">
+        <x:v>wrap de carne y cheddar x 210g froodie</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="str">
+        <x:v>wrap de jyq x 210g froodie</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="str">
+        <x:v>wrap de vegetales x 210g froodie</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="str">
+        <x:v>hamburguesa 80 gr frizzio</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="str">
+        <x:v>papas baston frizzio 720 gr</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2" t="str">
+        <x:v>pollo al disco c vegetales frizzio</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="str">
+        <x:v>tarta calabaza frizzio 175 gr</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="str">
+        <x:v>tarta espinaca frizzio 175 gr</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="str">
+        <x:v>tarta jamon y queso frizzio 175 gr</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="str">
+        <x:v>helado de agua</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="str">
+        <x:v>palito doble crunch</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="str">
+        <x:v>tentacion cadbury chocolate con almendras</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="str">
+        <x:v>tentacion cadbury yog frutilla</x:v>
+      </x:c>
+      <x:c r="B37" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="str">
+        <x:v>tentacion pina al agua</x:v>
+      </x:c>
+      <x:c r="B38" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2" t="str">
+        <x:v>torta primavera</x:v>
+      </x:c>
+      <x:c r="B39" s="2" t="str">
+        <x:v>Omitido por operación</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="2" t="str">
+        <x:v>canelones de carne 450 gr platos listos frizzio desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B40" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="2" t="str">
+        <x:v>empanada carne desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B41" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="2" t="str">
+        <x:v>empanada jamon y queso desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B42" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2" t="str">
+        <x:v>lasagna bolognesa con jamon y queso desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B43" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2" t="str">
+        <x:v>lasagna crema espinaca desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B44" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2" t="str">
+        <x:v>muslito a la portuguesa 400 gr platos listos frizzio desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B45" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2" t="str">
+        <x:v>pastel de papas 400 gr platos listos frizzio desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B46" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2" t="str">
+        <x:v>suprema napolitana c pure 450 gr platos listos frizzio desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B47" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="str">
+        <x:v>helado sin azucar chocolate desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B48" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="str">
+        <x:v>helado sin azucar frutilla a la crema display desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B49" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2" t="str">
+        <x:v>helado sin azucar frutilla a la crema desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B50" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="2" t="str">
+        <x:v>helado sin azucar crema durazno desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B51" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2" t="str">
+        <x:v>helado sin azucar chocolate display desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B52" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="2" t="str">
+        <x:v>helado sin azucar crema durazno display desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B53" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="2" t="str">
+        <x:v>yogurt helado frutilla sin tacc desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B54" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="2" t="str">
+        <x:v>yogurt helado frutos bosque sin tacc desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B55" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="2" t="str">
+        <x:v>yogurt helado mango maracuya sin tacc desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B56" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="2" t="str">
+        <x:v>palito pico dulce desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B57" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="2" t="str">
+        <x:v>alfajor shot desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B58" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="2" t="str">
+        <x:v>display postre vegano chocolate desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B59" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="2" t="str">
+        <x:v>display postre vegano mani desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B60" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="2" t="str">
+        <x:v>display postre vegano vainilla desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B61" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="2" t="str">
+        <x:v>postre cremoso cheesecake desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B62" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="2" t="str">
+        <x:v>postre cremoso chocolate desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B63" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="2" t="str">
+        <x:v>postre cremoso de frutilla desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B64" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="2" t="str">
+        <x:v>postre cremoso lemon pie desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B65" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="2" t="str">
+        <x:v>postre cremoso tiramisu desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B66" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="2" t="str">
+        <x:v>postre vegano chocolate desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B67" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="2" t="str">
+        <x:v>postre vegano mani desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B68" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="2" t="str">
+        <x:v>postre vegano vainilla desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B69" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="2" t="str">
+        <x:v>torta desactivado 23 02 2026</x:v>
+      </x:c>
+      <x:c r="B70" s="2" t="str">
+        <x:v>Desactivado: omitir siempre</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5583c85c7d34705"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec8a5dd290f4616"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Labs 2.2.0 - actualizar Maestro (2026-10-28 12:48:06 UTC)
</commit_message>
<xml_diff>
--- a/data/Maestro_Productos_Grido.xlsx
+++ b/data/Maestro_Productos_Grido.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" r:id="R747e6d6964c24753"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliases" sheetId="2" r:id="Rb0507c26604d42a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusiones" sheetId="3" r:id="R7789cc705f72416f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="Rddf0d05bc2d94fa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="5" r:id="R3d919bdf8b4b479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Productos" sheetId="1" r:id="Rf54aee9354e94e7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliases" sheetId="2" r:id="R23bd639ca22b4ff2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusiones" sheetId="3" r:id="Rfe81082f941b40ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="R1f6ff0f0134041c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuración" sheetId="5" r:id="R7c6f4ffdc11a421b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2861,13 +2861,15 @@
       <x:c r="E52" s="2" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="F52" s="2" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G52" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="H52" s="2"/>
+      <x:c r="F52" s="2" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="G52" s="2" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="H52" s="2" t="str">
+        <x:v>Discontinuado; excluir de pedidos y análisis nuevos</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="15" customHeight="1">
       <x:c r="A53" s="2" t="s">
@@ -3933,6 +3935,32 @@
       </x:c>
       <x:c r="H96" s="2" t="str">
         <x:v>Agregado por nuevo Mix de Ventas</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>postre chocolate duo</x:v>
+      </x:c>
+      <x:c r="B97" t="n">
+        <x:v>4000998</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>PACK 6 U. POSTRE CHOCOLATE DUO GR</x:v>
+      </x:c>
+      <x:c r="D97" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>Producto cerrado</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Sí</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>Producto nuevo. Datos de compra confirmados 27/10/2026.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3951,7 +3979,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19704c9ed6704e68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d8b255e59864489"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11041,6 +11069,60 @@
         <x:v>Preparado para venta individual</x:v>
       </x:c>
     </x:row>
+    <x:row r="271">
+      <x:c r="A271" t="str">
+        <x:v>Postre Chocolate Duo</x:v>
+      </x:c>
+      <x:c r="B271" t="str">
+        <x:v>postre chocolate duo</x:v>
+      </x:c>
+      <x:c r="C271" t="str">
+        <x:v>Producto cerrado</x:v>
+      </x:c>
+      <x:c r="D271"/>
+      <x:c r="E271" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F271" t="str">
+        <x:v>Stock</x:v>
+      </x:c>
+      <x:c r="G271" t="str">
+        <x:v>Postres</x:v>
+      </x:c>
+      <x:c r="H271" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I271" t="str">
+        <x:v>Código 4000998; pack x6 confirmado</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="272">
+      <x:c r="A272" t="str">
+        <x:v>Postre Chocolate Duo</x:v>
+      </x:c>
+      <x:c r="B272" t="str">
+        <x:v>postre chocolate duo</x:v>
+      </x:c>
+      <x:c r="C272" t="str">
+        <x:v>Producto cerrado</x:v>
+      </x:c>
+      <x:c r="D272"/>
+      <x:c r="E272" t="str">
+        <x:v>cantidad</x:v>
+      </x:c>
+      <x:c r="F272" t="str">
+        <x:v>Ventas data</x:v>
+      </x:c>
+      <x:c r="G272" t="str">
+        <x:v>Postres</x:v>
+      </x:c>
+      <x:c r="H272" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="I272" t="str">
+        <x:v>Código 4000998; pack x6 confirmado</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="H2:H216">
     <x:cfRule type="expression" dxfId="1" priority="1">
@@ -11057,7 +11139,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79ba85ba15ed49cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab9e30aff0384549"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11630,10 +11712,26 @@
         <x:v>Desactivado: omitir siempre</x:v>
       </x:c>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>seleccion argentina</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>Sabor discontinuado; excluir</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>Selección Argentina 7,800 Kg - Grido</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>Sabor discontinuado; excluir</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec8a5dd290f4616"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbd710dd84414e9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>